<commit_message>
replaced healthcare data rerun it
</commit_message>
<xml_diff>
--- a/cert-data/Healthcare-Certification-Report-10.05.2026.xlsx
+++ b/cert-data/Healthcare-Certification-Report-10.05.2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://konicaminoltanam-my.sharepoint.com/personal/rnesimi_kmbsus_com/Documents/Dashboard Reports/Healthcare Dashboard Reports/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{23E38052-4C84-4868-8D5A-623F8C77662D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{450F71E5-756C-4074-8E65-6FF5CF08E4DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DC5E560D-579C-485D-825F-94F306B9108B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1179" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1180" uniqueCount="291">
   <si>
     <t>User</t>
   </si>
@@ -4389,9 +4389,18 @@
       <c r="Q33" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="R33" s="9"/>
-      <c r="T33" s="11" t="s">
-        <v>40</v>
+      <c r="R33" s="9">
+        <v>46300</v>
+      </c>
+      <c r="S33" s="1" t="str">
+        <f>"FY"&amp;YEAR(R33)-IF(MONTH(R33)&lt;4,1,0)&amp;" "&amp;CHOOSE(MATCH(MONTH(R33),{1,4,7,10}),"Q4","Q1","Q2","Q3")</f>
+        <v>FY2026 Q3</v>
+      </c>
+      <c r="T33" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="U33" s="4" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="34" spans="1:21">

</xml_diff>